<commit_message>
chore: monthly GLOBALG.A.P certificate scrape 2026-08-07
</commit_message>
<xml_diff>
--- a/GGAP certificates latest.xlsx
+++ b/GGAP certificates latest.xlsx
@@ -410,8 +410,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="CertData" displayName="CertData" ref="A1:F99" headerRowCount="1">
-  <autoFilter ref="A1:F99"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="CertData" displayName="CertData" ref="A1:F100" headerRowCount="1">
+  <autoFilter ref="A1:F100"/>
   <tableColumns count="6">
     <tableColumn id="1" name="GGN"/>
     <tableColumn id="2" name="Producer Name"/>
@@ -740,7 +740,7 @@
         </is>
       </c>
       <c r="C3" s="3" t="n">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="E3" s="2" t="inlineStr">
         <is>
@@ -1218,11 +1218,11 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Blueberry</t>
+          <t>Tomato</t>
         </is>
       </c>
       <c r="C14" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="15">
@@ -1233,7 +1233,7 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Spring onion</t>
+          <t>Blueberry</t>
         </is>
       </c>
       <c r="C15" t="n">
@@ -1248,7 +1248,7 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Tomato</t>
+          <t>Spring onion</t>
         </is>
       </c>
       <c r="C16" t="n">
@@ -2470,52 +2470,48 @@
     <row r="82">
       <c r="A82" t="inlineStr">
         <is>
-          <t>Basil (herb)</t>
+          <t>Tomato</t>
         </is>
       </c>
       <c r="B82" t="inlineStr">
         <is>
-          <t>Lithuania</t>
+          <t>Latvia</t>
         </is>
       </c>
       <c r="C82" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t>Basil (herb)</t>
+          <t>Tomato</t>
         </is>
       </c>
       <c r="B83" t="inlineStr">
         <is>
-          <t>Latvia</t>
+          <t>Lithuania</t>
         </is>
       </c>
       <c r="C83" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="84">
       <c r="A84" t="inlineStr">
         <is>
-          <t>Basil (herb)</t>
-        </is>
-      </c>
-      <c r="B84" t="inlineStr">
-        <is>
-          <t>Estonia</t>
-        </is>
-      </c>
+          <t>Tomato</t>
+        </is>
+      </c>
+      <c r="B84" t="inlineStr"/>
       <c r="C84" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="85">
       <c r="A85" t="inlineStr">
         <is>
-          <t>Basil (herb)</t>
+          <t>Tomato</t>
         </is>
       </c>
       <c r="B85" t="inlineStr"/>
@@ -2526,7 +2522,7 @@
     <row r="86">
       <c r="A86" t="inlineStr">
         <is>
-          <t>Basil (herb)</t>
+          <t>Tomato</t>
         </is>
       </c>
       <c r="B86" t="inlineStr"/>
@@ -2537,7 +2533,7 @@
     <row r="87">
       <c r="A87" t="inlineStr">
         <is>
-          <t>Basil (herb)</t>
+          <t>Tomato</t>
         </is>
       </c>
       <c r="B87" t="inlineStr"/>
@@ -2548,7 +2544,7 @@
     <row r="88">
       <c r="A88" t="inlineStr">
         <is>
-          <t>Basil (herb)</t>
+          <t>Tomato</t>
         </is>
       </c>
       <c r="B88" t="inlineStr"/>
@@ -2559,7 +2555,7 @@
     <row r="89">
       <c r="A89" t="inlineStr">
         <is>
-          <t>Basil (herb)</t>
+          <t>Tomato</t>
         </is>
       </c>
       <c r="B89" t="inlineStr"/>
@@ -2570,7 +2566,7 @@
     <row r="90">
       <c r="A90" t="inlineStr">
         <is>
-          <t>Basil (herb)</t>
+          <t>Tomato</t>
         </is>
       </c>
       <c r="B90" t="inlineStr"/>
@@ -2581,7 +2577,7 @@
     <row r="91">
       <c r="A91" t="inlineStr">
         <is>
-          <t>Basil (herb)</t>
+          <t>Tomato</t>
         </is>
       </c>
       <c r="B91" t="inlineStr"/>
@@ -2592,12 +2588,12 @@
     <row r="92">
       <c r="A92" t="inlineStr">
         <is>
-          <t>Spring onion</t>
+          <t>Basil (herb)</t>
         </is>
       </c>
       <c r="B92" t="inlineStr">
         <is>
-          <t>Latvia</t>
+          <t>Lithuania</t>
         </is>
       </c>
       <c r="C92" t="n">
@@ -2607,33 +2603,37 @@
     <row r="93">
       <c r="A93" t="inlineStr">
         <is>
-          <t>Spring onion</t>
+          <t>Basil (herb)</t>
         </is>
       </c>
       <c r="B93" t="inlineStr">
         <is>
-          <t>Lithuania</t>
+          <t>Latvia</t>
         </is>
       </c>
       <c r="C93" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="94">
       <c r="A94" t="inlineStr">
         <is>
-          <t>Spring onion</t>
-        </is>
-      </c>
-      <c r="B94" t="inlineStr"/>
+          <t>Basil (herb)</t>
+        </is>
+      </c>
+      <c r="B94" t="inlineStr">
+        <is>
+          <t>Estonia</t>
+        </is>
+      </c>
       <c r="C94" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="95">
       <c r="A95" t="inlineStr">
         <is>
-          <t>Spring onion</t>
+          <t>Basil (herb)</t>
         </is>
       </c>
       <c r="B95" t="inlineStr"/>
@@ -2644,7 +2644,7 @@
     <row r="96">
       <c r="A96" t="inlineStr">
         <is>
-          <t>Spring onion</t>
+          <t>Basil (herb)</t>
         </is>
       </c>
       <c r="B96" t="inlineStr"/>
@@ -2655,7 +2655,7 @@
     <row r="97">
       <c r="A97" t="inlineStr">
         <is>
-          <t>Spring onion</t>
+          <t>Basil (herb)</t>
         </is>
       </c>
       <c r="B97" t="inlineStr"/>
@@ -2666,7 +2666,7 @@
     <row r="98">
       <c r="A98" t="inlineStr">
         <is>
-          <t>Spring onion</t>
+          <t>Basil (herb)</t>
         </is>
       </c>
       <c r="B98" t="inlineStr"/>
@@ -2677,7 +2677,7 @@
     <row r="99">
       <c r="A99" t="inlineStr">
         <is>
-          <t>Spring onion</t>
+          <t>Basil (herb)</t>
         </is>
       </c>
       <c r="B99" t="inlineStr"/>
@@ -2688,7 +2688,7 @@
     <row r="100">
       <c r="A100" t="inlineStr">
         <is>
-          <t>Spring onion</t>
+          <t>Basil (herb)</t>
         </is>
       </c>
       <c r="B100" t="inlineStr"/>
@@ -2699,7 +2699,7 @@
     <row r="101">
       <c r="A101" t="inlineStr">
         <is>
-          <t>Spring onion</t>
+          <t>Basil (herb)</t>
         </is>
       </c>
       <c r="B101" t="inlineStr"/>
@@ -2710,7 +2710,7 @@
     <row r="102">
       <c r="A102" t="inlineStr">
         <is>
-          <t>Tomato</t>
+          <t>Spring onion</t>
         </is>
       </c>
       <c r="B102" t="inlineStr">
@@ -2725,7 +2725,7 @@
     <row r="103">
       <c r="A103" t="inlineStr">
         <is>
-          <t>Tomato</t>
+          <t>Spring onion</t>
         </is>
       </c>
       <c r="B103" t="inlineStr">
@@ -2740,7 +2740,7 @@
     <row r="104">
       <c r="A104" t="inlineStr">
         <is>
-          <t>Tomato</t>
+          <t>Spring onion</t>
         </is>
       </c>
       <c r="B104" t="inlineStr"/>
@@ -2751,7 +2751,7 @@
     <row r="105">
       <c r="A105" t="inlineStr">
         <is>
-          <t>Tomato</t>
+          <t>Spring onion</t>
         </is>
       </c>
       <c r="B105" t="inlineStr"/>
@@ -2762,7 +2762,7 @@
     <row r="106">
       <c r="A106" t="inlineStr">
         <is>
-          <t>Tomato</t>
+          <t>Spring onion</t>
         </is>
       </c>
       <c r="B106" t="inlineStr"/>
@@ -2773,7 +2773,7 @@
     <row r="107">
       <c r="A107" t="inlineStr">
         <is>
-          <t>Tomato</t>
+          <t>Spring onion</t>
         </is>
       </c>
       <c r="B107" t="inlineStr"/>
@@ -2784,7 +2784,7 @@
     <row r="108">
       <c r="A108" t="inlineStr">
         <is>
-          <t>Tomato</t>
+          <t>Spring onion</t>
         </is>
       </c>
       <c r="B108" t="inlineStr"/>
@@ -2795,7 +2795,7 @@
     <row r="109">
       <c r="A109" t="inlineStr">
         <is>
-          <t>Tomato</t>
+          <t>Spring onion</t>
         </is>
       </c>
       <c r="B109" t="inlineStr"/>
@@ -2806,7 +2806,7 @@
     <row r="110">
       <c r="A110" t="inlineStr">
         <is>
-          <t>Tomato</t>
+          <t>Spring onion</t>
         </is>
       </c>
       <c r="B110" t="inlineStr"/>
@@ -2817,7 +2817,7 @@
     <row r="111">
       <c r="A111" t="inlineStr">
         <is>
-          <t>Tomato</t>
+          <t>Spring onion</t>
         </is>
       </c>
       <c r="B111" t="inlineStr"/>
@@ -5909,21 +5909,21 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Basil (herb)</t>
+          <t>Tomato</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Spring onion</t>
+          <t>Basil (herb)</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Tomato</t>
+          <t>Spring onion</t>
         </is>
       </c>
     </row>
@@ -6156,7 +6156,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>24</v>
+        <v>25</v>
       </c>
     </row>
     <row r="4">
@@ -6180,7 +6180,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F99"/>
+  <dimension ref="A1:F100"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -6930,17 +6930,17 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>4069453068148</t>
+          <t>4069453658271</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>ZS DIŽSKUDRAS</t>
+          <t>Latgales darzenu logisitka</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>Lecava - Bauskas novads</t>
+          <t>Tutāni</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
@@ -6962,17 +6962,17 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>4063651422405</t>
+          <t>4069453068148</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>SIA Mārupes siltumnīcas</t>
+          <t>ZS DIŽSKUDRAS</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>Jaunmārupe</t>
+          <t>Lecava - Bauskas novads</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
@@ -6994,22 +6994,22 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>4063651971187</t>
+          <t>4063651422405</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>Grüne Fee Eesti AS</t>
+          <t>SIA Mārupes siltumnīcas</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>Lohkva</t>
+          <t>Jaunmārupe</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>Estonia</t>
+          <t>Latvia</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
@@ -7019,24 +7019,24 @@
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>Basil (herb)</t>
+          <t>Tomato</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>4063651319316</t>
+          <t>4063651971187</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>Laheotsa OÜ</t>
+          <t>Grüne Fee Eesti AS</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>Harjumaa</t>
+          <t>Lohkva</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
@@ -7051,24 +7051,24 @@
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>Carrot</t>
+          <t>Basil (herb)</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>4063651971187</t>
+          <t>4063651319316</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>Grüne Fee Eesti AS</t>
+          <t>Laheotsa OÜ</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>Lohkva</t>
+          <t>Harjumaa</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
@@ -7083,7 +7083,7 @@
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t>Chive (herb)</t>
+          <t>Carrot</t>
         </is>
       </c>
     </row>
@@ -7115,7 +7115,7 @@
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>Coriander (herb)</t>
+          <t>Chive (herb)</t>
         </is>
       </c>
     </row>
@@ -7147,7 +7147,7 @@
       </c>
       <c r="F30" t="inlineStr">
         <is>
-          <t>Dill (herb)</t>
+          <t>Coriander (herb)</t>
         </is>
       </c>
     </row>
@@ -7179,7 +7179,7 @@
       </c>
       <c r="F31" t="inlineStr">
         <is>
-          <t>Lettuce</t>
+          <t>Dill (herb)</t>
         </is>
       </c>
     </row>
@@ -7211,7 +7211,7 @@
       </c>
       <c r="F32" t="inlineStr">
         <is>
-          <t>Oregano (herb)</t>
+          <t>Lettuce</t>
         </is>
       </c>
     </row>
@@ -7243,24 +7243,24 @@
       </c>
       <c r="F33" t="inlineStr">
         <is>
-          <t>Parsley (herb)</t>
+          <t>Oregano (herb)</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>4063651319316</t>
+          <t>4063651971187</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>Laheotsa OÜ</t>
+          <t>Grüne Fee Eesti AS</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>Harjumaa</t>
+          <t>Lohkva</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
@@ -7275,24 +7275,24 @@
       </c>
       <c r="F34" t="inlineStr">
         <is>
-          <t>Potato</t>
+          <t>Parsley (herb)</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>4063651316186</t>
+          <t>4063651319316</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>Simuna Remox OÜ</t>
+          <t>Laheotsa OÜ</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>Simuna</t>
+          <t>Harjumaa</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
@@ -7314,17 +7314,17 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>4063651704044</t>
+          <t>4063651316186</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>Kartuliait OÜ</t>
+          <t>Simuna Remox OÜ</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>Kambja</t>
+          <t>Simuna</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
@@ -7346,17 +7346,17 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>4063651971187</t>
+          <t>4063651704044</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>Grüne Fee Eesti AS</t>
+          <t>Kartuliait OÜ</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>Lohkva</t>
+          <t>Kambja</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
@@ -7371,7 +7371,7 @@
       </c>
       <c r="F37" t="inlineStr">
         <is>
-          <t>Spinach</t>
+          <t>Potato</t>
         </is>
       </c>
     </row>
@@ -7403,29 +7403,29 @@
       </c>
       <c r="F38" t="inlineStr">
         <is>
-          <t>Thyme (herb)</t>
+          <t>Spinach</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>4063651713169</t>
+          <t>4063651971187</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>UAB 'Naradava'</t>
+          <t>Grüne Fee Eesti AS</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>Pasvalio r.</t>
+          <t>Lohkva</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>Lithuania</t>
+          <t>Estonia</t>
         </is>
       </c>
       <c r="E39" t="inlineStr">
@@ -7435,24 +7435,24 @@
       </c>
       <c r="F39" t="inlineStr">
         <is>
-          <t>Apple</t>
+          <t>Thyme (herb)</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>4069453087842</t>
+          <t>4063651713169</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>Vitalijus Petronis</t>
+          <t>UAB 'Naradava'</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>Utenos apskritis</t>
+          <t>Pasvalio r.</t>
         </is>
       </c>
       <c r="D40" t="inlineStr">
@@ -7474,17 +7474,17 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>4063651916768</t>
+          <t>4069453087842</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>UAB Leafood</t>
+          <t>Vitalijus Petronis</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>Vilnius</t>
+          <t>Utenos apskritis</t>
         </is>
       </c>
       <c r="D41" t="inlineStr">
@@ -7499,24 +7499,24 @@
       </c>
       <c r="F41" t="inlineStr">
         <is>
-          <t>Arugula/Rocket (herb)</t>
+          <t>Apple</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>4063651942033</t>
+          <t>4063651916768</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>Irmos Šiaučiulienės ūkis</t>
+          <t>UAB Leafood</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>Marijampolės raj.</t>
+          <t>Vilnius</t>
         </is>
       </c>
       <c r="D42" t="inlineStr">
@@ -7531,24 +7531,24 @@
       </c>
       <c r="F42" t="inlineStr">
         <is>
-          <t>Asparagus</t>
+          <t>Arugula/Rocket (herb)</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>4063651916768</t>
+          <t>4063651942033</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>UAB Leafood</t>
+          <t>Irmos Šiaučiulienės ūkis</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>Vilnius</t>
+          <t>Marijampolės raj.</t>
         </is>
       </c>
       <c r="D43" t="inlineStr">
@@ -7563,24 +7563,24 @@
       </c>
       <c r="F43" t="inlineStr">
         <is>
-          <t>Baby leaf lettuce</t>
+          <t>Asparagus</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>4063061020512</t>
+          <t>4063651916768</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>UAB „Evaldo daržovės“/Evaldas Masevičius</t>
+          <t>UAB Leafood</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>Šalcininku r.</t>
+          <t>Vilnius</t>
         </is>
       </c>
       <c r="D44" t="inlineStr">
@@ -7595,7 +7595,7 @@
       </c>
       <c r="F44" t="inlineStr">
         <is>
-          <t>Baby leaf spinach</t>
+          <t>Baby leaf lettuce</t>
         </is>
       </c>
     </row>
@@ -7627,24 +7627,24 @@
       </c>
       <c r="F45" t="inlineStr">
         <is>
-          <t>Basil (herb)</t>
+          <t>Baby leaf spinach</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>4063651916768</t>
+          <t>4063061020512</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>UAB Leafood</t>
+          <t>UAB „Evaldo daržovės“/Evaldas Masevičius</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>Vilnius</t>
+          <t>Šalcininku r.</t>
         </is>
       </c>
       <c r="D46" t="inlineStr">
@@ -7666,17 +7666,17 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>4056186779229</t>
+          <t>4063651916768</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>ŽŪK Suvalkijos daržovės</t>
+          <t>UAB Leafood</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>Šakiu r.</t>
+          <t>Vilnius</t>
         </is>
       </c>
       <c r="D47" t="inlineStr">
@@ -7686,29 +7686,29 @@
       </c>
       <c r="E47" t="inlineStr">
         <is>
-          <t>Producer group</t>
+          <t>Producer</t>
         </is>
       </c>
       <c r="F47" t="inlineStr">
         <is>
-          <t>Beetroot</t>
+          <t>Basil (herb)</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>4069453329232</t>
+          <t>4056186779229</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>UAB Krekenava</t>
+          <t>ŽŪK Suvalkijos daržovės</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>Paneve?z?io raj.</t>
+          <t>Šakiu r.</t>
         </is>
       </c>
       <c r="D48" t="inlineStr">
@@ -7718,7 +7718,7 @@
       </c>
       <c r="E48" t="inlineStr">
         <is>
-          <t>Producer</t>
+          <t>Producer group</t>
         </is>
       </c>
       <c r="F48" t="inlineStr">
@@ -7730,17 +7730,17 @@
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>4056186833488</t>
+          <t>4069453329232</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>ŽŪK Jakiškiai</t>
+          <t>UAB Krekenava</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>Joniškio r. sav.</t>
+          <t>Paneve?z?io raj.</t>
         </is>
       </c>
       <c r="D49" t="inlineStr">
@@ -7762,17 +7762,17 @@
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>4059883732108</t>
+          <t>4056186833488</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>Ūkininkas Darius Matijošaitis</t>
+          <t>ŽŪK Jakiškiai</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>Vilkaviškio raj.</t>
+          <t>Joniškio r. sav.</t>
         </is>
       </c>
       <c r="D50" t="inlineStr">
@@ -7794,17 +7794,17 @@
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>4069453469464</t>
+          <t>4059883732108</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>Ūkininkas Aurimas Garlauskas</t>
+          <t>Ūkininkas Darius Matijošaitis</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>Pasvalio r.</t>
+          <t>Vilkaviškio raj.</t>
         </is>
       </c>
       <c r="D51" t="inlineStr">
@@ -7826,17 +7826,17 @@
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>4069453094574</t>
+          <t>4069453469464</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>Ūkininkė Justė Matijošaitienė</t>
+          <t>Ūkininkas Aurimas Garlauskas</t>
         </is>
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>Vilkaviškio r.,</t>
+          <t>Pasvalio r.</t>
         </is>
       </c>
       <c r="D52" t="inlineStr">
@@ -7858,17 +7858,17 @@
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>4059883253337</t>
+          <t>4069453094574</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>Ūkininkas Vidmantas Kvedaras</t>
+          <t>Ūkininkė Justė Matijošaitienė</t>
         </is>
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>Kedainiu dist.</t>
+          <t>Vilkaviškio r.,</t>
         </is>
       </c>
       <c r="D53" t="inlineStr">
@@ -7890,17 +7890,17 @@
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>4056186779212</t>
+          <t>4059883253337</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>UAB ALTA AGRO</t>
+          <t>Ūkininkas Vidmantas Kvedaras</t>
         </is>
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>Zarasai</t>
+          <t>Kedainiu dist.</t>
         </is>
       </c>
       <c r="D54" t="inlineStr">
@@ -7915,24 +7915,24 @@
       </c>
       <c r="F54" t="inlineStr">
         <is>
-          <t>Blueberry</t>
+          <t>Beetroot</t>
         </is>
       </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>4059883499193</t>
+          <t>4056186779212</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>U.A.B. Blueberrybaltic</t>
+          <t>UAB ALTA AGRO</t>
         </is>
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>Kaunatava Telsiai</t>
+          <t>Zarasai</t>
         </is>
       </c>
       <c r="D55" t="inlineStr">
@@ -7986,17 +7986,17 @@
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>4063651257762</t>
+          <t>4059883499193</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>Vitalija Morkūnienė</t>
+          <t>U.A.B. Blueberrybaltic</t>
         </is>
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>Pasvalys</t>
+          <t>Kaunatava Telsiai</t>
         </is>
       </c>
       <c r="D57" t="inlineStr">
@@ -8011,24 +8011,24 @@
       </c>
       <c r="F57" t="inlineStr">
         <is>
-          <t>Cabbage</t>
+          <t>Blueberry</t>
         </is>
       </c>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>4063651257748</t>
+          <t>4063651257762</t>
         </is>
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>Darius Morkūnas</t>
+          <t>Vitalija Morkūnienė</t>
         </is>
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>Daujėnų sen., Pasvalio r. sav.</t>
+          <t>Pasvalys</t>
         </is>
       </c>
       <c r="D58" t="inlineStr">
@@ -8050,17 +8050,17 @@
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>4063061958938</t>
+          <t>4063651257748</t>
         </is>
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>UAB Sodžiaus rytas</t>
+          <t>Darius Morkūnas</t>
         </is>
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>Pasvalio</t>
+          <t>Daujėnų sen., Pasvalio r. sav.</t>
         </is>
       </c>
       <c r="D59" t="inlineStr">
@@ -8082,17 +8082,17 @@
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>4059883253337</t>
+          <t>4063061958938</t>
         </is>
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>Ūkininkas Vidmantas Kvedaras</t>
+          <t>UAB Sodžiaus rytas</t>
         </is>
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>Kedainiu dist.</t>
+          <t>Pasvalio</t>
         </is>
       </c>
       <c r="D60" t="inlineStr">
@@ -8114,17 +8114,17 @@
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>4056186833488</t>
+          <t>4059883253337</t>
         </is>
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>ŽŪK Jakiškiai</t>
+          <t>Ūkininkas Vidmantas Kvedaras</t>
         </is>
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t>Joniškio r. sav.</t>
+          <t>Kedainiu dist.</t>
         </is>
       </c>
       <c r="D61" t="inlineStr">
@@ -8139,24 +8139,24 @@
       </c>
       <c r="F61" t="inlineStr">
         <is>
-          <t>Carrot</t>
+          <t>Cabbage</t>
         </is>
       </c>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>4063651257762</t>
+          <t>4056186833488</t>
         </is>
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>Vitalija Morkūnienė</t>
+          <t>ŽŪK Jakiškiai</t>
         </is>
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>Pasvalys</t>
+          <t>Joniškio r. sav.</t>
         </is>
       </c>
       <c r="D62" t="inlineStr">
@@ -8178,17 +8178,17 @@
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>4063651257748</t>
+          <t>4063651257762</t>
         </is>
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>Darius Morkūnas</t>
+          <t>Vitalija Morkūnienė</t>
         </is>
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>Daujėnų sen., Pasvalio r. sav.</t>
+          <t>Pasvalys</t>
         </is>
       </c>
       <c r="D63" t="inlineStr">
@@ -8210,17 +8210,17 @@
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>4063061958938</t>
+          <t>4063651257748</t>
         </is>
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>UAB Sodžiaus rytas</t>
+          <t>Darius Morkūnas</t>
         </is>
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>Pasvalio</t>
+          <t>Daujėnų sen., Pasvalio r. sav.</t>
         </is>
       </c>
       <c r="D64" t="inlineStr">
@@ -8242,17 +8242,17 @@
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>4063061177803</t>
+          <t>4063061958938</t>
         </is>
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>Ūkininkas Linas Šateika</t>
+          <t>UAB Sodžiaus rytas</t>
         </is>
       </c>
       <c r="C65" t="inlineStr">
         <is>
-          <t>Šiaulių r. sav.</t>
+          <t>Pasvalio</t>
         </is>
       </c>
       <c r="D65" t="inlineStr">
@@ -8274,17 +8274,17 @@
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>4059883253337</t>
+          <t>4063061177803</t>
         </is>
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>Ūkininkas Vidmantas Kvedaras</t>
+          <t>Ūkininkas Linas Šateika</t>
         </is>
       </c>
       <c r="C66" t="inlineStr">
         <is>
-          <t>Kedainiu dist.</t>
+          <t>Šiaulių r. sav.</t>
         </is>
       </c>
       <c r="D66" t="inlineStr">
@@ -8306,17 +8306,17 @@
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>4059883976991</t>
+          <t>4059883253337</t>
         </is>
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>Ūkininkas Vaidas Nagreckis</t>
+          <t>Ūkininkas Vidmantas Kvedaras</t>
         </is>
       </c>
       <c r="C67" t="inlineStr">
         <is>
-          <t>Raseiniu dist.</t>
+          <t>Kedainiu dist.</t>
         </is>
       </c>
       <c r="D67" t="inlineStr">
@@ -8331,24 +8331,24 @@
       </c>
       <c r="F67" t="inlineStr">
         <is>
-          <t>Celery</t>
+          <t>Carrot</t>
         </is>
       </c>
     </row>
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>4063651916768</t>
+          <t>4059883976991</t>
         </is>
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>UAB Leafood</t>
+          <t>Ūkininkas Vaidas Nagreckis</t>
         </is>
       </c>
       <c r="C68" t="inlineStr">
         <is>
-          <t>Vilnius</t>
+          <t>Raseiniu dist.</t>
         </is>
       </c>
       <c r="D68" t="inlineStr">
@@ -8363,24 +8363,24 @@
       </c>
       <c r="F68" t="inlineStr">
         <is>
-          <t>Coriander (herb)</t>
+          <t>Celery</t>
         </is>
       </c>
     </row>
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>4056186779229</t>
+          <t>4063651916768</t>
         </is>
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>ŽŪK Suvalkijos daržovės</t>
+          <t>UAB Leafood</t>
         </is>
       </c>
       <c r="C69" t="inlineStr">
         <is>
-          <t>Šakiu r.</t>
+          <t>Vilnius</t>
         </is>
       </c>
       <c r="D69" t="inlineStr">
@@ -8390,29 +8390,29 @@
       </c>
       <c r="E69" t="inlineStr">
         <is>
-          <t>Producer group</t>
+          <t>Producer</t>
         </is>
       </c>
       <c r="F69" t="inlineStr">
         <is>
-          <t>Courgette (zucchini, marrow)</t>
+          <t>Coriander (herb)</t>
         </is>
       </c>
     </row>
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>4069453223011</t>
+          <t>4056186779229</t>
         </is>
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>UAB Anykščių šiltnamiai</t>
+          <t>ŽŪK Suvalkijos daržovės</t>
         </is>
       </c>
       <c r="C70" t="inlineStr">
         <is>
-          <t>Vikonių k., Anykščių raj.</t>
+          <t>Šakiu r.</t>
         </is>
       </c>
       <c r="D70" t="inlineStr">
@@ -8422,29 +8422,29 @@
       </c>
       <c r="E70" t="inlineStr">
         <is>
-          <t>Producer</t>
+          <t>Producer group</t>
         </is>
       </c>
       <c r="F70" t="inlineStr">
         <is>
-          <t>Cucumber</t>
+          <t>Courgette (zucchini, marrow)</t>
         </is>
       </c>
     </row>
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>4063651931709</t>
+          <t>4069453223011</t>
         </is>
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>Ūkininkas Mantas Jasiukaitis</t>
+          <t>UAB Anykščių šiltnamiai</t>
         </is>
       </c>
       <c r="C71" t="inlineStr">
         <is>
-          <t>Radviliškio raj.</t>
+          <t>Vikonių k., Anykščių raj.</t>
         </is>
       </c>
       <c r="D71" t="inlineStr">
@@ -8466,17 +8466,17 @@
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
-          <t>4059883251395</t>
+          <t>4063651931709</t>
         </is>
       </c>
       <c r="B72" t="inlineStr">
         <is>
-          <t>UAB Agrošiltnamiai</t>
+          <t>Ūkininkas Mantas Jasiukaitis</t>
         </is>
       </c>
       <c r="C72" t="inlineStr">
         <is>
-          <t>Kedainiu dist.</t>
+          <t>Radviliškio raj.</t>
         </is>
       </c>
       <c r="D72" t="inlineStr">
@@ -8498,17 +8498,17 @@
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>4059883167955</t>
+          <t>4059883251395</t>
         </is>
       </c>
       <c r="B73" t="inlineStr">
         <is>
-          <t>UAB Kietaviskiu Gausa</t>
+          <t>UAB Agrošiltnamiai</t>
         </is>
       </c>
       <c r="C73" t="inlineStr">
         <is>
-          <t>Elektrenai</t>
+          <t>Kedainiu dist.</t>
         </is>
       </c>
       <c r="D73" t="inlineStr">
@@ -8530,17 +8530,17 @@
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>4063651643244</t>
+          <t>4059883167955</t>
         </is>
       </c>
       <c r="B74" t="inlineStr">
         <is>
-          <t>Ūkininkas Andrius Kavaliauskas</t>
+          <t>UAB Kietaviskiu Gausa</t>
         </is>
       </c>
       <c r="C74" t="inlineStr">
         <is>
-          <t>Radviliškio</t>
+          <t>Elektrenai</t>
         </is>
       </c>
       <c r="D74" t="inlineStr">
@@ -8562,17 +8562,17 @@
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>4059883976991</t>
+          <t>4063651643244</t>
         </is>
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>Ūkininkas Vaidas Nagreckis</t>
+          <t>Ūkininkas Andrius Kavaliauskas</t>
         </is>
       </c>
       <c r="C75" t="inlineStr">
         <is>
-          <t>Raseiniu dist.</t>
+          <t>Radviliškio</t>
         </is>
       </c>
       <c r="D75" t="inlineStr">
@@ -8587,24 +8587,24 @@
       </c>
       <c r="F75" t="inlineStr">
         <is>
-          <t>Lettuce</t>
+          <t>Cucumber</t>
         </is>
       </c>
     </row>
     <row r="76">
       <c r="A76" t="inlineStr">
         <is>
-          <t>4059883167955</t>
+          <t>4059883976991</t>
         </is>
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t>UAB Kietaviskiu Gausa</t>
+          <t>Ūkininkas Vaidas Nagreckis</t>
         </is>
       </c>
       <c r="C76" t="inlineStr">
         <is>
-          <t>Elektrenai</t>
+          <t>Raseiniu dist.</t>
         </is>
       </c>
       <c r="D76" t="inlineStr">
@@ -8626,17 +8626,17 @@
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>4063061020512</t>
+          <t>4059883167955</t>
         </is>
       </c>
       <c r="B77" t="inlineStr">
         <is>
-          <t>UAB „Evaldo daržovės“/Evaldas Masevičius</t>
+          <t>UAB Kietaviskiu Gausa</t>
         </is>
       </c>
       <c r="C77" t="inlineStr">
         <is>
-          <t>Šalcininku r.</t>
+          <t>Elektrenai</t>
         </is>
       </c>
       <c r="D77" t="inlineStr">
@@ -8658,17 +8658,17 @@
     <row r="78">
       <c r="A78" t="inlineStr">
         <is>
-          <t>4063651916768</t>
+          <t>4063061020512</t>
         </is>
       </c>
       <c r="B78" t="inlineStr">
         <is>
-          <t>UAB Leafood</t>
+          <t>UAB „Evaldo daržovės“/Evaldas Masevičius</t>
         </is>
       </c>
       <c r="C78" t="inlineStr">
         <is>
-          <t>Vilnius</t>
+          <t>Šalcininku r.</t>
         </is>
       </c>
       <c r="D78" t="inlineStr">
@@ -8683,24 +8683,24 @@
       </c>
       <c r="F78" t="inlineStr">
         <is>
-          <t>Mint (herb)</t>
+          <t>Lettuce</t>
         </is>
       </c>
     </row>
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t>4049929688988</t>
+          <t>4063651916768</t>
         </is>
       </c>
       <c r="B79" t="inlineStr">
         <is>
-          <t>Baltic Champs Ltd</t>
+          <t>UAB Leafood</t>
         </is>
       </c>
       <c r="C79" t="inlineStr">
         <is>
-          <t>Lietuva</t>
+          <t>Vilnius</t>
         </is>
       </c>
       <c r="D79" t="inlineStr">
@@ -8715,24 +8715,24 @@
       </c>
       <c r="F79" t="inlineStr">
         <is>
-          <t>Mushroom</t>
+          <t>Mint (herb)</t>
         </is>
       </c>
     </row>
     <row r="80">
       <c r="A80" t="inlineStr">
         <is>
-          <t>4063651931709</t>
+          <t>4049929688988</t>
         </is>
       </c>
       <c r="B80" t="inlineStr">
         <is>
-          <t>Ūkininkas Mantas Jasiukaitis</t>
+          <t>Baltic Champs Ltd</t>
         </is>
       </c>
       <c r="C80" t="inlineStr">
         <is>
-          <t>Radviliškio raj.</t>
+          <t>Lietuva</t>
         </is>
       </c>
       <c r="D80" t="inlineStr">
@@ -8747,24 +8747,24 @@
       </c>
       <c r="F80" t="inlineStr">
         <is>
-          <t>Onion</t>
+          <t>Mushroom</t>
         </is>
       </c>
     </row>
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>4063061125866</t>
+          <t>4063651931709</t>
         </is>
       </c>
       <c r="B81" t="inlineStr">
         <is>
-          <t>Vincentas Lataitis</t>
+          <t>Ūkininkas Mantas Jasiukaitis</t>
         </is>
       </c>
       <c r="C81" t="inlineStr">
         <is>
-          <t>Joniškis</t>
+          <t>Radviliškio raj.</t>
         </is>
       </c>
       <c r="D81" t="inlineStr">
@@ -8786,17 +8786,17 @@
     <row r="82">
       <c r="A82" t="inlineStr">
         <is>
-          <t>4056186779229</t>
+          <t>4063061125866</t>
         </is>
       </c>
       <c r="B82" t="inlineStr">
         <is>
-          <t>ŽŪK Suvalkijos daržovės</t>
+          <t>Vincentas Lataitis</t>
         </is>
       </c>
       <c r="C82" t="inlineStr">
         <is>
-          <t>Šakiu r.</t>
+          <t>Joniškis</t>
         </is>
       </c>
       <c r="D82" t="inlineStr">
@@ -8806,7 +8806,7 @@
       </c>
       <c r="E82" t="inlineStr">
         <is>
-          <t>Producer group</t>
+          <t>Producer</t>
         </is>
       </c>
       <c r="F82" t="inlineStr">
@@ -8818,17 +8818,17 @@
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t>4056186833488</t>
+          <t>4056186779229</t>
         </is>
       </c>
       <c r="B83" t="inlineStr">
         <is>
-          <t>ŽŪK Jakiškiai</t>
+          <t>ŽŪK Suvalkijos daržovės</t>
         </is>
       </c>
       <c r="C83" t="inlineStr">
         <is>
-          <t>Joniškio r. sav.</t>
+          <t>Šakiu r.</t>
         </is>
       </c>
       <c r="D83" t="inlineStr">
@@ -8838,7 +8838,7 @@
       </c>
       <c r="E83" t="inlineStr">
         <is>
-          <t>Producer</t>
+          <t>Producer group</t>
         </is>
       </c>
       <c r="F83" t="inlineStr">
@@ -8850,17 +8850,17 @@
     <row r="84">
       <c r="A84" t="inlineStr">
         <is>
-          <t>4063061177803</t>
+          <t>4056186833488</t>
         </is>
       </c>
       <c r="B84" t="inlineStr">
         <is>
-          <t>Ūkininkas Linas Šateika</t>
+          <t>ŽŪK Jakiškiai</t>
         </is>
       </c>
       <c r="C84" t="inlineStr">
         <is>
-          <t>Šiaulių r. sav.</t>
+          <t>Joniškio r. sav.</t>
         </is>
       </c>
       <c r="D84" t="inlineStr">
@@ -8882,17 +8882,17 @@
     <row r="85">
       <c r="A85" t="inlineStr">
         <is>
-          <t>4059883253337</t>
+          <t>4063061177803</t>
         </is>
       </c>
       <c r="B85" t="inlineStr">
         <is>
-          <t>Ūkininkas Vidmantas Kvedaras</t>
+          <t>Ūkininkas Linas Šateika</t>
         </is>
       </c>
       <c r="C85" t="inlineStr">
         <is>
-          <t>Kedainiu dist.</t>
+          <t>Šiaulių r. sav.</t>
         </is>
       </c>
       <c r="D85" t="inlineStr">
@@ -8914,17 +8914,17 @@
     <row r="86">
       <c r="A86" t="inlineStr">
         <is>
-          <t>4069453087842</t>
+          <t>4059883253337</t>
         </is>
       </c>
       <c r="B86" t="inlineStr">
         <is>
-          <t>Vitalijus Petronis</t>
+          <t>Ūkininkas Vidmantas Kvedaras</t>
         </is>
       </c>
       <c r="C86" t="inlineStr">
         <is>
-          <t>Utenos apskritis</t>
+          <t>Kedainiu dist.</t>
         </is>
       </c>
       <c r="D86" t="inlineStr">
@@ -8939,24 +8939,24 @@
       </c>
       <c r="F86" t="inlineStr">
         <is>
-          <t>Pear</t>
+          <t>Onion</t>
         </is>
       </c>
     </row>
     <row r="87">
       <c r="A87" t="inlineStr">
         <is>
-          <t>4056186779229</t>
+          <t>4069453087842</t>
         </is>
       </c>
       <c r="B87" t="inlineStr">
         <is>
-          <t>ŽŪK Suvalkijos daržovės</t>
+          <t>Vitalijus Petronis</t>
         </is>
       </c>
       <c r="C87" t="inlineStr">
         <is>
-          <t>Šakiu r.</t>
+          <t>Utenos apskritis</t>
         </is>
       </c>
       <c r="D87" t="inlineStr">
@@ -8966,29 +8966,29 @@
       </c>
       <c r="E87" t="inlineStr">
         <is>
-          <t>Producer group</t>
+          <t>Producer</t>
         </is>
       </c>
       <c r="F87" t="inlineStr">
         <is>
-          <t>Potato</t>
+          <t>Pear</t>
         </is>
       </c>
     </row>
     <row r="88">
       <c r="A88" t="inlineStr">
         <is>
-          <t>4059883732108</t>
+          <t>4056186779229</t>
         </is>
       </c>
       <c r="B88" t="inlineStr">
         <is>
-          <t>Ūkininkas Darius Matijošaitis</t>
+          <t>ŽŪK Suvalkijos daržovės</t>
         </is>
       </c>
       <c r="C88" t="inlineStr">
         <is>
-          <t>Vilkaviškio raj.</t>
+          <t>Šakiu r.</t>
         </is>
       </c>
       <c r="D88" t="inlineStr">
@@ -8998,7 +8998,7 @@
       </c>
       <c r="E88" t="inlineStr">
         <is>
-          <t>Producer</t>
+          <t>Producer group</t>
         </is>
       </c>
       <c r="F88" t="inlineStr">
@@ -9010,17 +9010,17 @@
     <row r="89">
       <c r="A89" t="inlineStr">
         <is>
-          <t>4069453094574</t>
+          <t>4059883732108</t>
         </is>
       </c>
       <c r="B89" t="inlineStr">
         <is>
-          <t>Ūkininkė Justė Matijošaitienė</t>
+          <t>Ūkininkas Darius Matijošaitis</t>
         </is>
       </c>
       <c r="C89" t="inlineStr">
         <is>
-          <t>Vilkaviškio r.,</t>
+          <t>Vilkaviškio raj.</t>
         </is>
       </c>
       <c r="D89" t="inlineStr">
@@ -9042,17 +9042,17 @@
     <row r="90">
       <c r="A90" t="inlineStr">
         <is>
-          <t>4059883253337</t>
+          <t>4069453094574</t>
         </is>
       </c>
       <c r="B90" t="inlineStr">
         <is>
-          <t>Ūkininkas Vidmantas Kvedaras</t>
+          <t>Ūkininkė Justė Matijošaitienė</t>
         </is>
       </c>
       <c r="C90" t="inlineStr">
         <is>
-          <t>Kedainiu dist.</t>
+          <t>Vilkaviškio r.,</t>
         </is>
       </c>
       <c r="D90" t="inlineStr">
@@ -9074,17 +9074,17 @@
     <row r="91">
       <c r="A91" t="inlineStr">
         <is>
-          <t>4056186779229</t>
+          <t>4059883253337</t>
         </is>
       </c>
       <c r="B91" t="inlineStr">
         <is>
-          <t>ŽŪK Suvalkijos daržovės</t>
+          <t>Ūkininkas Vidmantas Kvedaras</t>
         </is>
       </c>
       <c r="C91" t="inlineStr">
         <is>
-          <t>Šakiu r.</t>
+          <t>Kedainiu dist.</t>
         </is>
       </c>
       <c r="D91" t="inlineStr">
@@ -9094,29 +9094,29 @@
       </c>
       <c r="E91" t="inlineStr">
         <is>
-          <t>Producer group</t>
+          <t>Producer</t>
         </is>
       </c>
       <c r="F91" t="inlineStr">
         <is>
-          <t>Pumpkin</t>
+          <t>Potato</t>
         </is>
       </c>
     </row>
     <row r="92">
       <c r="A92" t="inlineStr">
         <is>
-          <t>4063061843937</t>
+          <t>4056186779229</t>
         </is>
       </c>
       <c r="B92" t="inlineStr">
         <is>
-          <t>JSC DEHIDRA</t>
+          <t>ŽŪK Suvalkijos daržovės</t>
         </is>
       </c>
       <c r="C92" t="inlineStr">
         <is>
-          <t>Sirvintos district</t>
+          <t>Šakiu r.</t>
         </is>
       </c>
       <c r="D92" t="inlineStr">
@@ -9126,29 +9126,29 @@
       </c>
       <c r="E92" t="inlineStr">
         <is>
-          <t>Producer</t>
+          <t>Producer group</t>
         </is>
       </c>
       <c r="F92" t="inlineStr">
         <is>
-          <t>Raspberry</t>
+          <t>Pumpkin</t>
         </is>
       </c>
     </row>
     <row r="93">
       <c r="A93" t="inlineStr">
         <is>
-          <t>4059883976991</t>
+          <t>4063061843937</t>
         </is>
       </c>
       <c r="B93" t="inlineStr">
         <is>
-          <t>Ūkininkas Vaidas Nagreckis</t>
+          <t>JSC DEHIDRA</t>
         </is>
       </c>
       <c r="C93" t="inlineStr">
         <is>
-          <t>Raseiniu dist.</t>
+          <t>Sirvintos district</t>
         </is>
       </c>
       <c r="D93" t="inlineStr">
@@ -9163,24 +9163,24 @@
       </c>
       <c r="F93" t="inlineStr">
         <is>
-          <t>Romaine/Cos lettuce</t>
+          <t>Raspberry</t>
         </is>
       </c>
     </row>
     <row r="94">
       <c r="A94" t="inlineStr">
         <is>
-          <t>4063651931709</t>
+          <t>4059883976991</t>
         </is>
       </c>
       <c r="B94" t="inlineStr">
         <is>
-          <t>Ūkininkas Mantas Jasiukaitis</t>
+          <t>Ūkininkas Vaidas Nagreckis</t>
         </is>
       </c>
       <c r="C94" t="inlineStr">
         <is>
-          <t>Radviliškio raj.</t>
+          <t>Raseiniu dist.</t>
         </is>
       </c>
       <c r="D94" t="inlineStr">
@@ -9195,24 +9195,24 @@
       </c>
       <c r="F94" t="inlineStr">
         <is>
-          <t>Spring onion</t>
+          <t>Romaine/Cos lettuce</t>
         </is>
       </c>
     </row>
     <row r="95">
       <c r="A95" t="inlineStr">
         <is>
-          <t>4063061020512</t>
+          <t>4063651931709</t>
         </is>
       </c>
       <c r="B95" t="inlineStr">
         <is>
-          <t>UAB „Evaldo daržovės“/Evaldas Masevičius</t>
+          <t>Ūkininkas Mantas Jasiukaitis</t>
         </is>
       </c>
       <c r="C95" t="inlineStr">
         <is>
-          <t>Šalcininku r.</t>
+          <t>Radviliškio raj.</t>
         </is>
       </c>
       <c r="D95" t="inlineStr">
@@ -9234,17 +9234,17 @@
     <row r="96">
       <c r="A96" t="inlineStr">
         <is>
-          <t>4063061843937</t>
+          <t>4063061020512</t>
         </is>
       </c>
       <c r="B96" t="inlineStr">
         <is>
-          <t>JSC DEHIDRA</t>
+          <t>UAB „Evaldo daržovės“/Evaldas Masevičius</t>
         </is>
       </c>
       <c r="C96" t="inlineStr">
         <is>
-          <t>Sirvintos district</t>
+          <t>Šalcininku r.</t>
         </is>
       </c>
       <c r="D96" t="inlineStr">
@@ -9259,24 +9259,24 @@
       </c>
       <c r="F96" t="inlineStr">
         <is>
-          <t>Strawberry</t>
+          <t>Spring onion</t>
         </is>
       </c>
     </row>
     <row r="97">
       <c r="A97" t="inlineStr">
         <is>
-          <t>4063651916768</t>
+          <t>4063061843937</t>
         </is>
       </c>
       <c r="B97" t="inlineStr">
         <is>
-          <t>UAB Leafood</t>
+          <t>JSC DEHIDRA</t>
         </is>
       </c>
       <c r="C97" t="inlineStr">
         <is>
-          <t>Vilnius</t>
+          <t>Sirvintos district</t>
         </is>
       </c>
       <c r="D97" t="inlineStr">
@@ -9291,24 +9291,24 @@
       </c>
       <c r="F97" t="inlineStr">
         <is>
-          <t>Thyme (herb)</t>
+          <t>Strawberry</t>
         </is>
       </c>
     </row>
     <row r="98">
       <c r="A98" t="inlineStr">
         <is>
-          <t>4069453223011</t>
+          <t>4063651916768</t>
         </is>
       </c>
       <c r="B98" t="inlineStr">
         <is>
-          <t>UAB Anykščių šiltnamiai</t>
+          <t>UAB Leafood</t>
         </is>
       </c>
       <c r="C98" t="inlineStr">
         <is>
-          <t>Vikonių k., Anykščių raj.</t>
+          <t>Vilnius</t>
         </is>
       </c>
       <c r="D98" t="inlineStr">
@@ -9323,37 +9323,69 @@
       </c>
       <c r="F98" t="inlineStr">
         <is>
-          <t>Tomato</t>
+          <t>Thyme (herb)</t>
         </is>
       </c>
     </row>
     <row r="99">
       <c r="A99" t="inlineStr">
         <is>
+          <t>4069453223011</t>
+        </is>
+      </c>
+      <c r="B99" t="inlineStr">
+        <is>
+          <t>UAB Anykščių šiltnamiai</t>
+        </is>
+      </c>
+      <c r="C99" t="inlineStr">
+        <is>
+          <t>Vikonių k., Anykščių raj.</t>
+        </is>
+      </c>
+      <c r="D99" t="inlineStr">
+        <is>
+          <t>Lithuania</t>
+        </is>
+      </c>
+      <c r="E99" t="inlineStr">
+        <is>
+          <t>Producer</t>
+        </is>
+      </c>
+      <c r="F99" t="inlineStr">
+        <is>
+          <t>Tomato</t>
+        </is>
+      </c>
+    </row>
+    <row r="100">
+      <c r="A100" t="inlineStr">
+        <is>
           <t>4059883167955</t>
         </is>
       </c>
-      <c r="B99" t="inlineStr">
+      <c r="B100" t="inlineStr">
         <is>
           <t>UAB Kietaviskiu Gausa</t>
         </is>
       </c>
-      <c r="C99" t="inlineStr">
+      <c r="C100" t="inlineStr">
         <is>
           <t>Elektrenai</t>
         </is>
       </c>
-      <c r="D99" t="inlineStr">
-        <is>
-          <t>Lithuania</t>
-        </is>
-      </c>
-      <c r="E99" t="inlineStr">
+      <c r="D100" t="inlineStr">
+        <is>
+          <t>Lithuania</t>
+        </is>
+      </c>
+      <c r="E100" t="inlineStr">
         <is>
           <t>Producer</t>
         </is>
       </c>
-      <c r="F99" t="inlineStr">
+      <c r="F100" t="inlineStr">
         <is>
           <t>Tomato</t>
         </is>

</xml_diff>